<commit_message>
updated foodbook to atlas alimentaire
</commit_message>
<xml_diff>
--- a/app-public/www/exposure_template.xlsx
+++ b/app-public/www/exposure_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://022gc-my.sharepoint.com/personal/megan_tooby2_phac-aspc_gc_ca/Documents/Desktop/Data sets/phac-foodbook-shiny-app/app-public/www/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19E4EA60-21D9-405F-9287-DF20ED6C1786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{19E4EA60-21D9-405F-9287-DF20ED6C1786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8DFCC9A-0AE6-4ED9-9478-96083E51E17D}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C807FD21-811A-4856-A172-CDC804D7645C}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11235" xr2:uid="{C807FD21-811A-4856-A172-CDC804D7645C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1111,9 +1111,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1301CF78-5E0B-4E9A-BA6B-3893EA60C19C}">
   <dimension ref="A1:E225"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1130,15 +1130,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -1147,15 +1147,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -1164,7 +1164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1172,7 +1172,7 @@
         <v>0</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -1181,7 +1181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -1198,7 +1198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1206,7 +1206,7 @@
         <v>0</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -1215,7 +1215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1223,7 +1223,7 @@
         <v>0</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1240,7 +1240,7 @@
         <v>0</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -1249,7 +1249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>0</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -1266,7 +1266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -1274,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -1283,7 +1283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -1291,7 +1291,7 @@
         <v>0</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11">
         <v>0</v>
@@ -1300,7 +1300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -1308,7 +1308,7 @@
         <v>0</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -1317,7 +1317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -1325,7 +1325,7 @@
         <v>0</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -1334,7 +1334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -1342,7 +1342,7 @@
         <v>0</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -1351,7 +1351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -1376,7 +1376,7 @@
         <v>0</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16">
         <v>0</v>
@@ -1385,7 +1385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -1393,7 +1393,7 @@
         <v>0</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17">
         <v>0</v>
@@ -1402,7 +1402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -1410,7 +1410,7 @@
         <v>0</v>
       </c>
       <c r="C18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -1419,7 +1419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -1427,7 +1427,7 @@
         <v>0</v>
       </c>
       <c r="C19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19">
         <v>0</v>
@@ -1436,7 +1436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -1444,7 +1444,7 @@
         <v>0</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -1453,7 +1453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -1461,7 +1461,7 @@
         <v>0</v>
       </c>
       <c r="C21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21">
         <v>0</v>
@@ -1470,7 +1470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -1478,7 +1478,7 @@
         <v>0</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -1487,7 +1487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -1495,7 +1495,7 @@
         <v>0</v>
       </c>
       <c r="C23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -1504,7 +1504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -1512,7 +1512,7 @@
         <v>0</v>
       </c>
       <c r="C24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D24">
         <v>0</v>
@@ -1521,7 +1521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>28</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>0</v>
       </c>
       <c r="C25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -1538,7 +1538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>29</v>
       </c>
@@ -1546,7 +1546,7 @@
         <v>0</v>
       </c>
       <c r="C26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26">
         <v>0</v>
@@ -1555,7 +1555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -1563,7 +1563,7 @@
         <v>0</v>
       </c>
       <c r="C27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -1572,7 +1572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>31</v>
       </c>
@@ -1580,7 +1580,7 @@
         <v>0</v>
       </c>
       <c r="C28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28">
         <v>0</v>
@@ -1589,7 +1589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>32</v>
       </c>
@@ -1597,7 +1597,7 @@
         <v>0</v>
       </c>
       <c r="C29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29">
         <v>0</v>
@@ -1606,7 +1606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>33</v>
       </c>
@@ -1614,7 +1614,7 @@
         <v>0</v>
       </c>
       <c r="C30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -1623,7 +1623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -1631,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="C31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -1640,7 +1640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>35</v>
       </c>
@@ -1648,7 +1648,7 @@
         <v>0</v>
       </c>
       <c r="C32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -1657,7 +1657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>36</v>
       </c>
@@ -1665,7 +1665,7 @@
         <v>0</v>
       </c>
       <c r="C33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D33">
         <v>0</v>
@@ -1674,7 +1674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>37</v>
       </c>
@@ -1682,7 +1682,7 @@
         <v>0</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34">
         <v>0</v>
@@ -1691,7 +1691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>38</v>
       </c>
@@ -1699,7 +1699,7 @@
         <v>0</v>
       </c>
       <c r="C35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D35">
         <v>0</v>
@@ -1708,7 +1708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>39</v>
       </c>
@@ -1716,7 +1716,7 @@
         <v>0</v>
       </c>
       <c r="C36">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D36">
         <v>0</v>
@@ -1725,7 +1725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>40</v>
       </c>
@@ -1733,7 +1733,7 @@
         <v>0</v>
       </c>
       <c r="C37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D37">
         <v>0</v>
@@ -1742,7 +1742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>41</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>0</v>
       </c>
       <c r="C38">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38">
         <v>0</v>
@@ -1759,7 +1759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>42</v>
       </c>
@@ -1767,7 +1767,7 @@
         <v>0</v>
       </c>
       <c r="C39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D39">
         <v>0</v>
@@ -1776,7 +1776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>43</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>0</v>
       </c>
       <c r="C40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D40">
         <v>0</v>
@@ -1793,7 +1793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>44</v>
       </c>
@@ -1801,7 +1801,7 @@
         <v>0</v>
       </c>
       <c r="C41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D41">
         <v>0</v>
@@ -1810,7 +1810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>45</v>
       </c>
@@ -1818,7 +1818,7 @@
         <v>0</v>
       </c>
       <c r="C42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D42">
         <v>0</v>
@@ -1827,7 +1827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>46</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>0</v>
       </c>
       <c r="C43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43">
         <v>0</v>
@@ -1844,7 +1844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>47</v>
       </c>
@@ -1852,7 +1852,7 @@
         <v>0</v>
       </c>
       <c r="C44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D44">
         <v>0</v>
@@ -1861,7 +1861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>48</v>
       </c>
@@ -1869,7 +1869,7 @@
         <v>0</v>
       </c>
       <c r="C45">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D45">
         <v>0</v>
@@ -1878,7 +1878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>49</v>
       </c>
@@ -1886,7 +1886,7 @@
         <v>0</v>
       </c>
       <c r="C46">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D46">
         <v>0</v>
@@ -1895,7 +1895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>50</v>
       </c>
@@ -1903,7 +1903,7 @@
         <v>0</v>
       </c>
       <c r="C47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D47">
         <v>0</v>
@@ -1912,7 +1912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>51</v>
       </c>
@@ -1920,7 +1920,7 @@
         <v>0</v>
       </c>
       <c r="C48">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D48">
         <v>0</v>
@@ -1929,7 +1929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>52</v>
       </c>
@@ -1937,7 +1937,7 @@
         <v>0</v>
       </c>
       <c r="C49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D49">
         <v>0</v>
@@ -1946,7 +1946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>53</v>
       </c>
@@ -1954,7 +1954,7 @@
         <v>0</v>
       </c>
       <c r="C50">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D50">
         <v>0</v>
@@ -1963,7 +1963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>54</v>
       </c>
@@ -1971,7 +1971,7 @@
         <v>0</v>
       </c>
       <c r="C51">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D51">
         <v>0</v>
@@ -1980,7 +1980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>55</v>
       </c>
@@ -1988,7 +1988,7 @@
         <v>0</v>
       </c>
       <c r="C52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D52">
         <v>0</v>
@@ -1997,7 +1997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>56</v>
       </c>
@@ -2005,7 +2005,7 @@
         <v>0</v>
       </c>
       <c r="C53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D53">
         <v>0</v>
@@ -2014,7 +2014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>57</v>
       </c>
@@ -2022,7 +2022,7 @@
         <v>0</v>
       </c>
       <c r="C54">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D54">
         <v>0</v>
@@ -2031,7 +2031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>58</v>
       </c>
@@ -2039,7 +2039,7 @@
         <v>0</v>
       </c>
       <c r="C55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D55">
         <v>0</v>
@@ -2048,7 +2048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>59</v>
       </c>
@@ -2056,7 +2056,7 @@
         <v>0</v>
       </c>
       <c r="C56">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D56">
         <v>0</v>
@@ -2065,7 +2065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>60</v>
       </c>
@@ -2073,7 +2073,7 @@
         <v>0</v>
       </c>
       <c r="C57">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D57">
         <v>0</v>
@@ -2082,7 +2082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>61</v>
       </c>
@@ -2090,7 +2090,7 @@
         <v>0</v>
       </c>
       <c r="C58">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D58">
         <v>0</v>
@@ -2099,7 +2099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>62</v>
       </c>
@@ -2107,7 +2107,7 @@
         <v>0</v>
       </c>
       <c r="C59">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D59">
         <v>0</v>
@@ -2116,7 +2116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>63</v>
       </c>
@@ -2124,7 +2124,7 @@
         <v>0</v>
       </c>
       <c r="C60">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D60">
         <v>0</v>
@@ -2133,7 +2133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>64</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>0</v>
       </c>
       <c r="C61">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D61">
         <v>0</v>
@@ -2150,7 +2150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>65</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>0</v>
       </c>
       <c r="C62">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D62">
         <v>0</v>
@@ -2167,7 +2167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>66</v>
       </c>
@@ -2175,7 +2175,7 @@
         <v>0</v>
       </c>
       <c r="C63">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D63">
         <v>0</v>
@@ -2184,7 +2184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>67</v>
       </c>
@@ -2192,7 +2192,7 @@
         <v>0</v>
       </c>
       <c r="C64">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D64">
         <v>0</v>
@@ -2201,7 +2201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>68</v>
       </c>
@@ -2209,7 +2209,7 @@
         <v>0</v>
       </c>
       <c r="C65">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D65">
         <v>0</v>
@@ -2218,7 +2218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>69</v>
       </c>
@@ -2226,7 +2226,7 @@
         <v>0</v>
       </c>
       <c r="C66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D66">
         <v>0</v>
@@ -2235,7 +2235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>70</v>
       </c>
@@ -2243,7 +2243,7 @@
         <v>0</v>
       </c>
       <c r="C67">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D67">
         <v>0</v>
@@ -2252,7 +2252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>71</v>
       </c>
@@ -2260,7 +2260,7 @@
         <v>0</v>
       </c>
       <c r="C68">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D68">
         <v>0</v>
@@ -2269,7 +2269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>72</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>0</v>
       </c>
       <c r="C69">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D69">
         <v>0</v>
@@ -2286,7 +2286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>73</v>
       </c>
@@ -2294,7 +2294,7 @@
         <v>0</v>
       </c>
       <c r="C70">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D70">
         <v>0</v>
@@ -2303,7 +2303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>74</v>
       </c>
@@ -2311,7 +2311,7 @@
         <v>0</v>
       </c>
       <c r="C71">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D71">
         <v>0</v>
@@ -2320,7 +2320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>75</v>
       </c>
@@ -2328,7 +2328,7 @@
         <v>0</v>
       </c>
       <c r="C72">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D72">
         <v>0</v>
@@ -2337,7 +2337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>76</v>
       </c>
@@ -2345,7 +2345,7 @@
         <v>0</v>
       </c>
       <c r="C73">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D73">
         <v>0</v>
@@ -2354,7 +2354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>77</v>
       </c>
@@ -2362,7 +2362,7 @@
         <v>0</v>
       </c>
       <c r="C74">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D74">
         <v>0</v>
@@ -2371,7 +2371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>78</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>0</v>
       </c>
       <c r="C75">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D75">
         <v>0</v>
@@ -2388,7 +2388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>79</v>
       </c>
@@ -2396,7 +2396,7 @@
         <v>0</v>
       </c>
       <c r="C76">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D76">
         <v>0</v>
@@ -2405,7 +2405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>80</v>
       </c>
@@ -2413,7 +2413,7 @@
         <v>0</v>
       </c>
       <c r="C77">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D77">
         <v>0</v>
@@ -2422,7 +2422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>81</v>
       </c>
@@ -2430,7 +2430,7 @@
         <v>0</v>
       </c>
       <c r="C78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D78">
         <v>0</v>
@@ -2439,7 +2439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>82</v>
       </c>
@@ -2447,7 +2447,7 @@
         <v>0</v>
       </c>
       <c r="C79">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D79">
         <v>0</v>
@@ -2456,7 +2456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>83</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>0</v>
       </c>
       <c r="C80">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D80">
         <v>0</v>
@@ -2473,7 +2473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>84</v>
       </c>
@@ -2481,7 +2481,7 @@
         <v>0</v>
       </c>
       <c r="C81">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D81">
         <v>0</v>
@@ -2490,7 +2490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>85</v>
       </c>
@@ -2498,7 +2498,7 @@
         <v>0</v>
       </c>
       <c r="C82">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D82">
         <v>0</v>
@@ -2507,7 +2507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>86</v>
       </c>
@@ -2515,7 +2515,7 @@
         <v>0</v>
       </c>
       <c r="C83">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D83">
         <v>0</v>
@@ -2524,7 +2524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>87</v>
       </c>
@@ -2532,7 +2532,7 @@
         <v>0</v>
       </c>
       <c r="C84">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D84">
         <v>0</v>
@@ -2541,7 +2541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>88</v>
       </c>
@@ -2549,7 +2549,7 @@
         <v>0</v>
       </c>
       <c r="C85">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D85">
         <v>0</v>
@@ -2558,7 +2558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>89</v>
       </c>
@@ -2566,7 +2566,7 @@
         <v>0</v>
       </c>
       <c r="C86">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D86">
         <v>0</v>
@@ -2575,7 +2575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>90</v>
       </c>
@@ -2583,7 +2583,7 @@
         <v>0</v>
       </c>
       <c r="C87">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D87">
         <v>0</v>
@@ -2592,7 +2592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>91</v>
       </c>
@@ -2600,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="C88">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D88">
         <v>0</v>
@@ -2609,7 +2609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>92</v>
       </c>
@@ -2617,7 +2617,7 @@
         <v>0</v>
       </c>
       <c r="C89">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D89">
         <v>0</v>
@@ -2626,7 +2626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>93</v>
       </c>
@@ -2634,7 +2634,7 @@
         <v>0</v>
       </c>
       <c r="C90">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D90">
         <v>0</v>
@@ -2643,7 +2643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>94</v>
       </c>
@@ -2651,7 +2651,7 @@
         <v>0</v>
       </c>
       <c r="C91">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D91">
         <v>0</v>
@@ -2660,7 +2660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>95</v>
       </c>
@@ -2668,7 +2668,7 @@
         <v>0</v>
       </c>
       <c r="C92">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D92">
         <v>0</v>
@@ -2677,7 +2677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>96</v>
       </c>
@@ -2685,7 +2685,7 @@
         <v>0</v>
       </c>
       <c r="C93">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D93">
         <v>0</v>
@@ -2694,7 +2694,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>97</v>
       </c>
@@ -2702,7 +2702,7 @@
         <v>0</v>
       </c>
       <c r="C94">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D94">
         <v>0</v>
@@ -2711,7 +2711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>98</v>
       </c>
@@ -2719,7 +2719,7 @@
         <v>0</v>
       </c>
       <c r="C95">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D95">
         <v>0</v>
@@ -2728,7 +2728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>99</v>
       </c>
@@ -2736,7 +2736,7 @@
         <v>0</v>
       </c>
       <c r="C96">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D96">
         <v>0</v>
@@ -2745,7 +2745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>100</v>
       </c>
@@ -2753,7 +2753,7 @@
         <v>0</v>
       </c>
       <c r="C97">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D97">
         <v>0</v>
@@ -2762,7 +2762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>101</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>0</v>
       </c>
       <c r="C98">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D98">
         <v>0</v>
@@ -2779,7 +2779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>102</v>
       </c>
@@ -2787,7 +2787,7 @@
         <v>0</v>
       </c>
       <c r="C99">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D99">
         <v>0</v>
@@ -2796,7 +2796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>103</v>
       </c>
@@ -2804,7 +2804,7 @@
         <v>0</v>
       </c>
       <c r="C100">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D100">
         <v>0</v>
@@ -2813,7 +2813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>104</v>
       </c>
@@ -2821,7 +2821,7 @@
         <v>0</v>
       </c>
       <c r="C101">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D101">
         <v>0</v>
@@ -2830,7 +2830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>105</v>
       </c>
@@ -2838,7 +2838,7 @@
         <v>0</v>
       </c>
       <c r="C102">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D102">
         <v>0</v>
@@ -2847,7 +2847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>106</v>
       </c>
@@ -2855,7 +2855,7 @@
         <v>0</v>
       </c>
       <c r="C103">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D103">
         <v>0</v>
@@ -2864,7 +2864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>107</v>
       </c>
@@ -2881,7 +2881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>108</v>
       </c>
@@ -2898,7 +2898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>109</v>
       </c>
@@ -2915,7 +2915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>110</v>
       </c>
@@ -2932,12 +2932,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>111</v>
       </c>
       <c r="B108">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C108">
         <v>0</v>
@@ -2949,12 +2949,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>112</v>
       </c>
       <c r="B109">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C109">
         <v>0</v>
@@ -2966,12 +2966,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>113</v>
       </c>
       <c r="B110">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C110">
         <v>0</v>
@@ -2983,12 +2983,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>114</v>
       </c>
       <c r="B111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C111">
         <v>0</v>
@@ -3000,12 +3000,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>115</v>
       </c>
       <c r="B112">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C112">
         <v>0</v>
@@ -3017,12 +3017,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>116</v>
       </c>
       <c r="B113">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C113">
         <v>0</v>
@@ -3034,12 +3034,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>117</v>
       </c>
       <c r="B114">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C114">
         <v>0</v>
@@ -3051,12 +3051,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>118</v>
       </c>
       <c r="B115">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C115">
         <v>0</v>
@@ -3068,12 +3068,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>119</v>
       </c>
       <c r="B116">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C116">
         <v>0</v>
@@ -3085,12 +3085,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>120</v>
       </c>
       <c r="B117">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C117">
         <v>0</v>
@@ -3102,12 +3102,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>121</v>
       </c>
       <c r="B118">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C118">
         <v>0</v>
@@ -3119,12 +3119,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>122</v>
       </c>
       <c r="B119">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C119">
         <v>0</v>
@@ -3136,12 +3136,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>123</v>
       </c>
       <c r="B120">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C120">
         <v>0</v>
@@ -3153,12 +3153,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>124</v>
       </c>
       <c r="B121">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C121">
         <v>0</v>
@@ -3170,12 +3170,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>125</v>
       </c>
       <c r="B122">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C122">
         <v>0</v>
@@ -3187,12 +3187,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>126</v>
       </c>
       <c r="B123">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C123">
         <v>0</v>
@@ -3204,12 +3204,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>127</v>
       </c>
       <c r="B124">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C124">
         <v>0</v>
@@ -3221,12 +3221,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>128</v>
       </c>
       <c r="B125">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C125">
         <v>0</v>
@@ -3238,12 +3238,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>129</v>
       </c>
       <c r="B126">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C126">
         <v>0</v>
@@ -3255,12 +3255,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>130</v>
       </c>
       <c r="B127">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C127">
         <v>0</v>
@@ -3272,12 +3272,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>131</v>
       </c>
       <c r="B128">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="C128">
         <v>0</v>
@@ -3289,12 +3289,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>132</v>
       </c>
       <c r="B129">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C129">
         <v>0</v>
@@ -3306,12 +3306,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>133</v>
       </c>
       <c r="B130">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C130">
         <v>0</v>
@@ -3323,12 +3323,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>134</v>
       </c>
       <c r="B131">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="C131">
         <v>0</v>
@@ -3340,12 +3340,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>135</v>
       </c>
       <c r="B132">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C132">
         <v>0</v>
@@ -3357,12 +3357,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>136</v>
       </c>
       <c r="B133">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C133">
         <v>0</v>
@@ -3374,12 +3374,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>137</v>
       </c>
       <c r="B134">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C134">
         <v>0</v>
@@ -3391,12 +3391,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>138</v>
       </c>
       <c r="B135">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C135">
         <v>0</v>
@@ -3408,12 +3408,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>139</v>
       </c>
       <c r="B136">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C136">
         <v>0</v>
@@ -3425,12 +3425,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>140</v>
       </c>
       <c r="B137">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C137">
         <v>0</v>
@@ -3442,12 +3442,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>141</v>
       </c>
       <c r="B138">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C138">
         <v>0</v>
@@ -3459,12 +3459,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>142</v>
       </c>
       <c r="B139">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C139">
         <v>0</v>
@@ -3476,12 +3476,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>143</v>
       </c>
       <c r="B140">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C140">
         <v>0</v>
@@ -3493,12 +3493,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>144</v>
       </c>
       <c r="B141">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C141">
         <v>0</v>
@@ -3510,12 +3510,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>145</v>
       </c>
       <c r="B142">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="C142">
         <v>0</v>
@@ -3527,114 +3527,114 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>146</v>
       </c>
       <c r="B143">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C143">
         <v>0</v>
       </c>
       <c r="D143">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E143">
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>147</v>
       </c>
       <c r="B144">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C144">
         <v>0</v>
       </c>
       <c r="D144">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E144">
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>148</v>
       </c>
       <c r="B145">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C145">
         <v>0</v>
       </c>
       <c r="D145">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E145">
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>149</v>
       </c>
       <c r="B146">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C146">
         <v>0</v>
       </c>
       <c r="D146">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E146">
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>150</v>
       </c>
       <c r="B147">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C147">
         <v>0</v>
       </c>
       <c r="D147">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E147">
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>151</v>
       </c>
       <c r="B148">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C148">
         <v>0</v>
       </c>
       <c r="D148">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E148">
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>152</v>
       </c>
       <c r="B149">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C149">
         <v>0</v>
@@ -3646,29 +3646,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>153</v>
       </c>
       <c r="B150">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C150">
         <v>0</v>
       </c>
       <c r="D150">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E150">
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>154</v>
       </c>
       <c r="B151">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C151">
         <v>0</v>
@@ -3680,29 +3680,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>155</v>
       </c>
       <c r="B152">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C152">
         <v>0</v>
       </c>
       <c r="D152">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E152">
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>156</v>
       </c>
       <c r="B153">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C153">
         <v>0</v>
@@ -3714,80 +3714,80 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>157</v>
       </c>
       <c r="B154">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C154">
         <v>0</v>
       </c>
       <c r="D154">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E154">
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>158</v>
       </c>
       <c r="B155">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C155">
         <v>0</v>
       </c>
       <c r="D155">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E155">
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>159</v>
       </c>
       <c r="B156">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C156">
         <v>0</v>
       </c>
       <c r="D156">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E156">
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>160</v>
       </c>
       <c r="B157">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C157">
         <v>0</v>
       </c>
       <c r="D157">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E157">
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>161</v>
       </c>
       <c r="B158">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C158">
         <v>0</v>
@@ -3799,100 +3799,100 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>162</v>
       </c>
       <c r="B159">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C159">
         <v>0</v>
       </c>
       <c r="D159">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E159">
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>163</v>
       </c>
       <c r="B160">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C160">
         <v>0</v>
       </c>
       <c r="D160">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E160">
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>164</v>
       </c>
       <c r="B161">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C161">
         <v>0</v>
       </c>
       <c r="D161">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E161">
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>165</v>
       </c>
       <c r="B162">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C162">
         <v>0</v>
       </c>
       <c r="D162">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E162">
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>166</v>
       </c>
       <c r="B163">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C163">
         <v>0</v>
       </c>
       <c r="D163">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E163">
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>167</v>
       </c>
       <c r="B164">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C164">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D164">
         <v>0</v>
@@ -3901,15 +3901,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>168</v>
       </c>
       <c r="B165">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C165">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D165">
         <v>0</v>
@@ -3918,24 +3918,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>169</v>
       </c>
       <c r="B166">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C166">
         <v>0</v>
       </c>
       <c r="D166">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E166">
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>170</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>171</v>
       </c>
@@ -3969,7 +3969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>172</v>
       </c>
@@ -3986,7 +3986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>173</v>
       </c>
@@ -4003,7 +4003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>174</v>
       </c>
@@ -4020,7 +4020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>175</v>
       </c>
@@ -4037,7 +4037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>176</v>
       </c>
@@ -4054,7 +4054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>177</v>
       </c>
@@ -4071,7 +4071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>178</v>
       </c>
@@ -4088,7 +4088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>179</v>
       </c>
@@ -4105,7 +4105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>180</v>
       </c>
@@ -4122,7 +4122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>181</v>
       </c>
@@ -4139,7 +4139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>182</v>
       </c>
@@ -4156,7 +4156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>183</v>
       </c>
@@ -4173,7 +4173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>184</v>
       </c>
@@ -4190,7 +4190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>185</v>
       </c>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>186</v>
       </c>
@@ -4224,7 +4224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>187</v>
       </c>
@@ -4241,7 +4241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>188</v>
       </c>
@@ -4258,7 +4258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>189</v>
       </c>
@@ -4275,7 +4275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>190</v>
       </c>
@@ -4292,7 +4292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>191</v>
       </c>
@@ -4309,7 +4309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>192</v>
       </c>
@@ -4326,7 +4326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>193</v>
       </c>
@@ -4343,7 +4343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>194</v>
       </c>
@@ -4360,7 +4360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>195</v>
       </c>
@@ -4377,7 +4377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>196</v>
       </c>
@@ -4394,7 +4394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>197</v>
       </c>
@@ -4411,7 +4411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>198</v>
       </c>
@@ -4428,7 +4428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>199</v>
       </c>
@@ -4445,7 +4445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>200</v>
       </c>
@@ -4462,7 +4462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>201</v>
       </c>
@@ -4479,7 +4479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>202</v>
       </c>
@@ -4496,7 +4496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>203</v>
       </c>
@@ -4513,7 +4513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>204</v>
       </c>
@@ -4530,7 +4530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>205</v>
       </c>
@@ -4547,7 +4547,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>206</v>
       </c>
@@ -4564,7 +4564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>207</v>
       </c>
@@ -4581,7 +4581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>208</v>
       </c>
@@ -4598,7 +4598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>209</v>
       </c>
@@ -4615,7 +4615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>210</v>
       </c>
@@ -4632,7 +4632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>211</v>
       </c>
@@ -4649,7 +4649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>212</v>
       </c>
@@ -4666,7 +4666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>213</v>
       </c>
@@ -4683,7 +4683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>214</v>
       </c>
@@ -4700,7 +4700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>215</v>
       </c>
@@ -4717,7 +4717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>216</v>
       </c>
@@ -4734,7 +4734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>217</v>
       </c>
@@ -4751,7 +4751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>218</v>
       </c>
@@ -4768,7 +4768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>219</v>
       </c>
@@ -4785,7 +4785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>220</v>
       </c>
@@ -4802,7 +4802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>221</v>
       </c>
@@ -4819,7 +4819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>222</v>
       </c>
@@ -4836,7 +4836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>223</v>
       </c>
@@ -4853,7 +4853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>224</v>
       </c>
@@ -4870,7 +4870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>225</v>
       </c>
@@ -4887,7 +4887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>226</v>
       </c>
@@ -4904,7 +4904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>227</v>
       </c>
@@ -4921,7 +4921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>228</v>
       </c>
@@ -4949,7 +4949,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF730949-E9F4-4C95-A136-02192A76D7E5}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -4961,7 +4961,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3A6D433-AE8E-4C63-9602-52BF04A00468}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -4971,6 +4971,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5a23a45f-f767-4528-886f-1c9bae1748ed" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BCF50380F26F9C4AB4316B881F1E0074" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="24f8853f2367eb3b6b7cf2cc2677425f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="a1c7653d-d0a9-4a9e-8039-9f6c7086724e" xmlns:ns4="5a23a45f-f767-4528-886f-1c9bae1748ed" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="421a08077b78c6bbcf5f73fdaeae6ea9" ns3:_="" ns4:_="">
     <xsd:import namespace="a1c7653d-d0a9-4a9e-8039-9f6c7086724e"/>
@@ -5223,24 +5240,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9F1F9B1-3B9B-42B1-B196-1820F7DE9321}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="a1c7653d-d0a9-4a9e-8039-9f6c7086724e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="5a23a45f-f767-4528-886f-1c9bae1748ed"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5a23a45f-f767-4528-886f-1c9bae1748ed" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5BBB2A38-2F9A-496A-A9F8-739D03A53A1E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02E72C6B-5122-45ED-8D87-B32092C24A59}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5257,29 +5282,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5BBB2A38-2F9A-496A-A9F8-739D03A53A1E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9F1F9B1-3B9B-42B1-B196-1820F7DE9321}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="a1c7653d-d0a9-4a9e-8039-9f6c7086724e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="5a23a45f-f767-4528-886f-1c9bae1748ed"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>